<commit_message>
Complete Resources workbook repairs and portable companion parity
Repair five existing workbooks without redesigning their layouts; restore corrected Export Check 1.2.0 and recover Family checklist metadata. Align human instructions, versions and portable JSON/CSV examples across all 13 packages. Preserve all licence notices and taxonomy machine files unchanged. Review branch only; no production or public-main promotion.

Verification: 13 Export Check scenarios; all five workbook ZIP/import/recalculation checks; 132 relative links; 10 companion format checks. Exact binary blob hashes verified before commit.
</commit_message>
<xml_diff>
--- a/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
+++ b/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
@@ -7,20 +7,20 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxonomy'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Taxonomy'!$A$1:$G$16</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,16 @@
       <b val="1"/>
       <color rgb="00000000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +55,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -75,6 +88,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -441,6 +463,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Household Records Filing Guide</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Open Household Records Taxonomy | Guide version 0.1.1 | 17 September 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Choose the main folder</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>File a record by what it is mainly about. Link to it from other relevant places. Keep backups and any copies you are required to keep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>A useful question</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Where would you look for this record when you need it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Keep insurance policies and claims in Insurance. A note or link can connect them to the home, vehicle, trip or pet they cover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Use the specific category</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Keep a lease in Home &amp; property, vehicle financing in Vehicles &amp; transportation, and an employment agreement in Employment &amp; income. Legal &amp; estate covers personal legal and estate matters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Insurance, work benefits or care?</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Insurance policy: Insurance. Work benefits enrolment: Employment &amp; income. Medication or care records: Health &amp; care.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>File format</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PDF, photo, email, spreadsheet or paper is not a category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Only use what you need</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>You do not need records in every category. Use the categories that help your household.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Protect personal information</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>The handling notes are practical reminders, not legal privacy classifications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>How long to keep records</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>A reminder to review a record is not a deletion date. Follow the applicable legal or tax requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>For software use</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Stable category IDs and technical fields are in taxonomy.json and taxonomy.csv. Their categories are unchanged by this guide update.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -454,37 +626,37 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>What belongs here</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Examples</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>When it applies</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Sensitivity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Review when</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Related areas</t>
         </is>
@@ -1049,154 +1221,4 @@
   <autoFilter ref="A1:G16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="105" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Open Household Records Taxonomy</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Human workbook — public review candidate 0.1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Core rule</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Give each record one primary home based on what it is mainly about. Keep other connections as relationships rather than duplicate primary copies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Retrieval test</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>If this record disappeared, which part of household life would notice first?</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Policies and claims live in Insurance even when they cover a home, vehicle, trip or pet. The covered subject remains a relationship.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Specific context first</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>A lease stays with Home &amp; property; vehicle financing with Vehicles &amp; transportation; an employment agreement with Employment &amp; income. Legal &amp; estate is for personal legal authority, status, representation, court or estate matters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Coverage vs care</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Insurance policy/coverage → Insurance. Employment-benefit enrolment/admin → Employment &amp; income. Medication, treatment, provider and care records → Health &amp; care.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>File format</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>PDF, photo, email, spreadsheet or paper is not a category.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Applicability</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>A category existing does not mean every household needs records in it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Sensitivity</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Sensitivity labels are practical handling cues, not legal/privacy classifications.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Retention</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Review triggers are not retention periods. Follow the relevant authority for legal or tax obligations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Machine data</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Stable IDs and technical fields are available in taxonomy.json / taxonomy.csv; this workbook is deliberately optimized for human reading.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Promote reconciled Resources artifacts to public main
Promote only the current Resources-owned companion files from the reviewed Resources branch. Normalize the repository landing page to production URLs. Preserve unrelated public-repository content and existing licence decisions.
</commit_message>
<xml_diff>
--- a/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
+++ b/taxonomies/open-household-records-taxonomy/taxonomy.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxonomy'!$A$1:$G$16</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -461,7 +461,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>What belongs here</t>
+          <t>What goes here</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -471,22 +471,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>When it applies</t>
+          <t>When to use it</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Sensitivity</t>
+          <t>Privacy notes</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Review when</t>
+          <t>When to update it</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Related areas</t>
+          <t>Related categories</t>
         </is>
       </c>
     </row>
@@ -1067,12 +1067,12 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Open Household Records Taxonomy</t>
+          <t>Household Records Filing Guide</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Human workbook — public review candidate 0.1.0</t>
+          <t>Human-readable guide, maintenance candidate 0.1.1. The formal reference is Open Household Records Taxonomy.</t>
         </is>
       </c>
     </row>
@@ -1084,19 +1084,19 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Give each record one primary home based on what it is mainly about. Keep other connections as relationships rather than duplicate primary copies.</t>
+          <t>Give each record a main home based on what it is mostly about. Add a note or link to other relevant categories. Keep backups and any copies you need.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Retrieval test</t>
+          <t>Where would you look?</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>If this record disappeared, which part of household life would notice first?</t>
+          <t>Think about where you would first look for this record when you need it.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Policies and claims live in Insurance even when they cover a home, vehicle, trip or pet. The covered subject remains a relationship.</t>
+          <t>Keep policies and claims in Insurance. Add a note about the home, vehicle, trip or pet they cover.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A lease stays with Home &amp; property; vehicle financing with Vehicles &amp; transportation; an employment agreement with Employment &amp; income. Legal &amp; estate is for personal legal authority, status, representation, court or estate matters.</t>
+          <t>Keep a home lease with Home &amp; property, vehicle financing with Vehicles &amp; transportation, and an employment agreement with Employment &amp; income. Use Legal &amp; estate for wills, powers of attorney, court matters and similar personal legal records.</t>
         </is>
       </c>
     </row>
@@ -1151,48 +1151,48 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Applicability</t>
+          <t>What applies</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>A category existing does not mean every household needs records in it.</t>
+          <t>Use the categories that help your household. You do not need a record in every category.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Sensitivity</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity labels are practical handling cues, not legal/privacy classifications.</t>
+          <t>The privacy notes are practical handling reminders, not legal classifications.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Retention</t>
+          <t>How long to keep records</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Review triggers are not retention periods. Follow the relevant authority for legal or tax obligations.</t>
+          <t>The update reminders are not deletion dates. Check the official requirements that apply before disposing of legal or tax records.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Machine data</t>
+          <t>Technical files</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Stable IDs and technical fields are available in taxonomy.json / taxonomy.csv; this workbook is deliberately optimized for human reading.</t>
+          <t>The package includes taxonomy.json and taxonomy.csv for people building software. This workbook is the human-readable guide. Reuse terms have not been assigned to the taxonomy; see LICENSE-NOTICE.md.</t>
         </is>
       </c>
     </row>

</xml_diff>